<commit_message>
Add report guidance and benchmark metrics
</commit_message>
<xml_diff>
--- a/reports/excel/optimized_portfolios.xlsx
+++ b/reports/excel/optimized_portfolios.xlsx
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5000000000000018</v>
+        <v>0.5000000000000058</v>
       </c>
     </row>
     <row r="3">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1499999999999988</v>
+        <v>0.1499999999999977</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1499999999999998</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="12">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1354996179024126</v>
+        <v>0.1358597379273871</v>
       </c>
     </row>
     <row r="3">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07372701822445404</v>
+        <v>0.07392356062289895</v>
       </c>
     </row>
     <row r="4">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04095108089677391</v>
+        <v>0.04129848856761442</v>
       </c>
     </row>
     <row r="5">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02357738483766925</v>
+        <v>0.02359095888798457</v>
       </c>
     </row>
     <row r="6">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01931037025710269</v>
+        <v>0.01933848868056387</v>
       </c>
     </row>
     <row r="7">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02808073014879975</v>
+        <v>0.02810783134564399</v>
       </c>
     </row>
     <row r="8">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0795676364091098</v>
+        <v>0.07945637154458751</v>
       </c>
     </row>
     <row r="9">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.07669500667584295</v>
+        <v>0.07658436309798122</v>
       </c>
     </row>
     <row r="10">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.003498787170287954</v>
+        <v>-0.004082492277633465</v>
       </c>
     </row>
     <row r="11">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1863748670627137</v>
+        <v>0.1868900671457263</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.02352371234328343</v>
+        <v>0.02346960388294939</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.04418790507949188</v>
+        <v>-0.04427055714493688</v>
       </c>
     </row>
   </sheetData>
@@ -781,40 +781,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.0306086811678833</v>
+        <v>0.03061055162907053</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02704848083700863</v>
+        <v>0.02705031270108093</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02716514934848669</v>
+        <v>0.02717108089842512</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003329224421194868</v>
+        <v>0.000333396862655863</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.001189955738383231</v>
+        <v>-0.001189442191261068</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0003849743640598883</v>
+        <v>-0.000384462676792857</v>
       </c>
       <c r="H2" t="n">
-        <v>0.001565980052617745</v>
+        <v>0.001567662776933946</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02590054344387245</v>
+        <v>0.02590033361957083</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01298895443157605</v>
+        <v>0.01298417150365833</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03338596900771639</v>
+        <v>0.03339183273804214</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006985233071542945</v>
+        <v>-0.006985008289441838</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0367737987603482</v>
+        <v>0.03677409985101048</v>
       </c>
     </row>
     <row r="3">
@@ -824,40 +824,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02704848083700863</v>
+        <v>0.02705031270108093</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03228104545551517</v>
+        <v>0.03228255425366702</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03078502076491787</v>
+        <v>0.03078926637774642</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0005144072538324381</v>
+        <v>0.0005147233710181068</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0009248909211351693</v>
+        <v>-0.0009245265702002489</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.786590499493595e-05</v>
+        <v>-2.749536005062632e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>0.004815049127311793</v>
+        <v>0.004815778593322297</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0243268085876282</v>
+        <v>0.02432640440575425</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01423905485230903</v>
+        <v>0.01423486301403834</v>
       </c>
       <c r="K3" t="n">
-        <v>0.02826461522262368</v>
+        <v>0.0282690508669</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.006924108830819272</v>
+        <v>-0.006924106176672476</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04051414849179754</v>
+        <v>0.04051413872263669</v>
       </c>
     </row>
     <row r="4">
@@ -867,40 +867,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02716514934848669</v>
+        <v>0.02717108089842512</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03078502076491787</v>
+        <v>0.03078926637774642</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0409532005240168</v>
+        <v>0.04096377209129554</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004483447416162975</v>
+        <v>0.0004490356898721208</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.000978144390821148</v>
+        <v>-0.0009772348987412891</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.182527853849557e-05</v>
+        <v>-1.092347514908783e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.005982316533663606</v>
+        <v>0.00598284375047626</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02348100095325859</v>
+        <v>0.02347948778986474</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01602979917334637</v>
+        <v>0.01601750702113731</v>
       </c>
       <c r="K4" t="n">
-        <v>0.02986958070833765</v>
+        <v>0.0298813022857886</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007008794819680837</v>
+        <v>-0.007009201483147245</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04655415004313663</v>
+        <v>0.04655339091380395</v>
       </c>
     </row>
     <row r="5">
@@ -910,40 +910,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0003329224421194868</v>
+        <v>0.000333396862655863</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005144072538324381</v>
+        <v>0.0005147233710181068</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0004483447416162975</v>
+        <v>0.0004490356898721208</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002543674852504231</v>
+        <v>0.00254370286938505</v>
       </c>
       <c r="F5" t="n">
-        <v>0.001482139695307435</v>
+        <v>0.00148218237588971</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002042182491791761</v>
+        <v>0.002042228304807083</v>
       </c>
       <c r="H5" t="n">
-        <v>0.002269239642028206</v>
+        <v>0.002269208916107364</v>
       </c>
       <c r="I5" t="n">
-        <v>0.002079965296540761</v>
+        <v>0.002079815580105561</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.0006999433048521711</v>
+        <v>-0.0007008118460263069</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0004795654059130041</v>
+        <v>0.0004803369407737381</v>
       </c>
       <c r="L5" t="n">
-        <v>0.005761367546447318</v>
+        <v>0.005761292209264112</v>
       </c>
       <c r="M5" t="n">
-        <v>3.998438256559361e-05</v>
+        <v>3.994710976774526e-05</v>
       </c>
     </row>
     <row r="6">
@@ -953,40 +953,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.001189955738383231</v>
+        <v>-0.001189442191261068</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.0009248909211351693</v>
+        <v>-0.0009245265702002489</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.000978144390821148</v>
+        <v>-0.0009772348987412891</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001482139695307435</v>
+        <v>0.00148218237588971</v>
       </c>
       <c r="F6" t="n">
-        <v>0.001536378130691438</v>
+        <v>0.001536449860786993</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001572246503788202</v>
+        <v>0.001572305482666053</v>
       </c>
       <c r="H6" t="n">
-        <v>0.001868420593947178</v>
+        <v>0.00186845068242548</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0003561198673624891</v>
+        <v>0.0003559723338068283</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.001184216757439315</v>
+        <v>-0.001185230637683308</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.001107648766157896</v>
+        <v>-0.001106653588632952</v>
       </c>
       <c r="L6" t="n">
-        <v>0.00436177054355946</v>
+        <v>0.004361708697666991</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.001505251109531347</v>
+        <v>-0.001505339436466972</v>
       </c>
     </row>
     <row r="7">
@@ -996,40 +996,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0003849743640598883</v>
+        <v>-0.000384462676792857</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.786590499493595e-05</v>
+        <v>-2.749536005062632e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.182527853849557e-05</v>
+        <v>-1.092347514908783e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002042182491791761</v>
+        <v>0.002042228304807083</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001572246503788202</v>
+        <v>0.001572305482666053</v>
       </c>
       <c r="G7" t="n">
-        <v>0.003392752280320046</v>
+        <v>0.003392818703741044</v>
       </c>
       <c r="H7" t="n">
-        <v>0.003051659166847742</v>
+        <v>0.003051702675547901</v>
       </c>
       <c r="I7" t="n">
-        <v>0.001394774960317419</v>
+        <v>0.00139464176020171</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0009348496496101919</v>
+        <v>0.0009338399556922046</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.0002791710782483401</v>
+        <v>-0.0002782008106463274</v>
       </c>
       <c r="L7" t="n">
-        <v>0.006216625695908984</v>
+        <v>0.006216564708259299</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001211761223016674</v>
+        <v>0.0001211401917078383</v>
       </c>
     </row>
     <row r="8">
@@ -1039,40 +1039,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001565980052617745</v>
+        <v>0.001567662776933946</v>
       </c>
       <c r="C8" t="n">
-        <v>0.004815049127311793</v>
+        <v>0.004815778593322297</v>
       </c>
       <c r="D8" t="n">
-        <v>0.005982316533663606</v>
+        <v>0.00598284375047626</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002269239642028206</v>
+        <v>0.002269208916107364</v>
       </c>
       <c r="F8" t="n">
-        <v>0.001868420593947178</v>
+        <v>0.00186845068242548</v>
       </c>
       <c r="G8" t="n">
-        <v>0.003051659166847742</v>
+        <v>0.003051702675547901</v>
       </c>
       <c r="H8" t="n">
-        <v>0.02727739965822988</v>
+        <v>0.02727611014739878</v>
       </c>
       <c r="I8" t="n">
-        <v>0.003577668779634077</v>
+        <v>0.003576973333025768</v>
       </c>
       <c r="J8" t="n">
-        <v>0.007498326128939696</v>
+        <v>0.007495680830096611</v>
       </c>
       <c r="K8" t="n">
-        <v>0.001881991604258652</v>
+        <v>0.001883252046567955</v>
       </c>
       <c r="L8" t="n">
-        <v>0.005267724154292097</v>
+        <v>0.005267248349672161</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01259485864313964</v>
+        <v>0.01259414405596525</v>
       </c>
     </row>
     <row r="9">
@@ -1082,40 +1082,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02590054344387245</v>
+        <v>0.02590033361957083</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0243268085876282</v>
+        <v>0.02432640440575425</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02348100095325859</v>
+        <v>0.02347948778986474</v>
       </c>
       <c r="E9" t="n">
-        <v>0.002079965296540761</v>
+        <v>0.002079815580105561</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003561198673624891</v>
+        <v>0.0003559723338068283</v>
       </c>
       <c r="G9" t="n">
-        <v>0.001394774960317419</v>
+        <v>0.00139464176020171</v>
       </c>
       <c r="H9" t="n">
-        <v>0.003577668779634077</v>
+        <v>0.003576973333025768</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03953340348155201</v>
+        <v>0.03953331932102008</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0097406365002063</v>
+        <v>0.009741445968415129</v>
       </c>
       <c r="K9" t="n">
-        <v>0.02463651482620324</v>
+        <v>0.02463516539174786</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.001700353501904926</v>
+        <v>-0.001700509511680643</v>
       </c>
       <c r="M9" t="n">
-        <v>0.03105434522384402</v>
+        <v>0.03105413838978375</v>
       </c>
     </row>
     <row r="10">
@@ -1125,40 +1125,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.01298895443157605</v>
+        <v>0.01298417150365833</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01423905485230903</v>
+        <v>0.01423486301403834</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01602979917334637</v>
+        <v>0.01601750702113731</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0006999433048521711</v>
+        <v>-0.0007008118460263069</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.001184216757439315</v>
+        <v>-0.001185230637683308</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0009348496496101919</v>
+        <v>0.0009338399556922046</v>
       </c>
       <c r="H10" t="n">
-        <v>0.007498326128939696</v>
+        <v>0.007495680830096611</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0097406365002063</v>
+        <v>0.009741445968415129</v>
       </c>
       <c r="J10" t="n">
-        <v>0.04458943211661513</v>
+        <v>0.0446006486456187</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01190559723340761</v>
+        <v>0.01189300389162079</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.006830467822581066</v>
+        <v>-0.006830686291870362</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02548633506151435</v>
+        <v>0.02548618581130556</v>
       </c>
     </row>
     <row r="11">
@@ -1168,40 +1168,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.03338596900771639</v>
+        <v>0.03339183273804214</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02826461522262368</v>
+        <v>0.0282690508669</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02986958070833765</v>
+        <v>0.0298813022857886</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0004795654059130041</v>
+        <v>0.0004803369407737381</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.001107648766157896</v>
+        <v>-0.001106653588632952</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0002791710782483401</v>
+        <v>-0.0002782008106463274</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001881991604258652</v>
+        <v>0.001883252046567955</v>
       </c>
       <c r="I11" t="n">
-        <v>0.02463651482620324</v>
+        <v>0.02463516539174786</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01190559723340761</v>
+        <v>0.01189300389162079</v>
       </c>
       <c r="K11" t="n">
-        <v>0.04273472595167611</v>
+        <v>0.04274739260848172</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.006334730128793119</v>
+        <v>-0.006334950366969848</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03972803676707876</v>
+        <v>0.03972757972848921</v>
       </c>
     </row>
     <row r="12">
@@ -1211,40 +1211,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.006985233071542945</v>
+        <v>-0.006985008289441838</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.006924108830819272</v>
+        <v>-0.006924106176672476</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.007008794819680837</v>
+        <v>-0.007009201483147245</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005761367546447318</v>
+        <v>0.005761292209264112</v>
       </c>
       <c r="F12" t="n">
-        <v>0.00436177054355946</v>
+        <v>0.004361708697666991</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006216625695908984</v>
+        <v>0.006216564708259299</v>
       </c>
       <c r="H12" t="n">
-        <v>0.005267724154292097</v>
+        <v>0.005267248349672161</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.001700353501904926</v>
+        <v>-0.001700509511680643</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.006830467822581066</v>
+        <v>-0.006830686291870362</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.006334730128793119</v>
+        <v>-0.006334950366969848</v>
       </c>
       <c r="L12" t="n">
-        <v>0.02237615639971379</v>
+        <v>0.0223760349350659</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.01025769506389224</v>
+        <v>-0.01025788740331246</v>
       </c>
     </row>
     <row r="13">
@@ -1254,40 +1254,40 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0367737987603482</v>
+        <v>0.03677409985101048</v>
       </c>
       <c r="C13" t="n">
-        <v>0.04051414849179754</v>
+        <v>0.04051413872263669</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04655415004313663</v>
+        <v>0.04655339091380395</v>
       </c>
       <c r="E13" t="n">
-        <v>3.998438256559361e-05</v>
+        <v>3.994710976774526e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.001505251109531347</v>
+        <v>-0.001505339436466972</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0001211761223016674</v>
+        <v>0.0001211401917078383</v>
       </c>
       <c r="H13" t="n">
-        <v>0.01259485864313964</v>
+        <v>0.01259414405596525</v>
       </c>
       <c r="I13" t="n">
-        <v>0.03105434522384402</v>
+        <v>0.03105413838978375</v>
       </c>
       <c r="J13" t="n">
-        <v>0.02548633506151435</v>
+        <v>0.02548618581130556</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03972803676707876</v>
+        <v>0.03972757972848921</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.01025769506389224</v>
+        <v>-0.01025788740331246</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1179569517676314</v>
+        <v>0.1179567242533223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add latest research pipeline updates
</commit_message>
<xml_diff>
--- a/reports/excel/optimized_portfolios.xlsx
+++ b/reports/excel/optimized_portfolios.xlsx
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5000000000000058</v>
+        <v>0.5000000000000009</v>
       </c>
     </row>
     <row r="3">
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000073</v>
       </c>
     </row>
     <row r="4">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1499999999999977</v>
+        <v>0.1499999999999996</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.15</v>
+        <v>0.1499999999999997</v>
       </c>
     </row>
     <row r="12">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1358597379273871</v>
+        <v>0.1358956347461182</v>
       </c>
     </row>
     <row r="3">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07392356062289895</v>
+        <v>0.0739750553109757</v>
       </c>
     </row>
     <row r="4">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04129848856761442</v>
+        <v>0.04133315844834007</v>
       </c>
     </row>
     <row r="5">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02359095888798457</v>
+        <v>0.0236045698975873</v>
       </c>
     </row>
     <row r="6">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01933848868056387</v>
+        <v>0.01934128567286342</v>
       </c>
     </row>
     <row r="7">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02810783134564399</v>
+        <v>0.02813492693711761</v>
       </c>
     </row>
     <row r="8">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.07945637154458751</v>
+        <v>0.07936883329785949</v>
       </c>
     </row>
     <row r="9">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.07658436309798122</v>
+        <v>0.07645137401388813</v>
       </c>
     </row>
     <row r="10">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.004082492277633465</v>
+        <v>-0.003438676536680951</v>
       </c>
     </row>
     <row r="11">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1868900671457263</v>
+        <v>0.1869328080968509</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.02346960388294939</v>
+        <v>0.02352762072477277</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.04427055714493688</v>
+        <v>-0.04413709254914255</v>
       </c>
     </row>
   </sheetData>
@@ -781,40 +781,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03061055162907053</v>
+        <v>0.03061090257805427</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02705031270108093</v>
+        <v>0.02705080294781807</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02717108089842512</v>
+        <v>0.02717185745198413</v>
       </c>
       <c r="E2" t="n">
-        <v>0.000333396862655863</v>
+        <v>0.0003335598448687919</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.001189442191261068</v>
+        <v>-0.001189382735895836</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.000384462676792857</v>
+        <v>-0.0003842762657988831</v>
       </c>
       <c r="H2" t="n">
-        <v>0.001567662776933946</v>
+        <v>0.00156736672673012</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02590033361957083</v>
+        <v>0.0258995946128974</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01298417150365833</v>
+        <v>0.01298748098504069</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03339183273804214</v>
+        <v>0.03339260737938018</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006985008289441838</v>
+        <v>-0.006984655662240311</v>
       </c>
       <c r="M2" t="n">
-        <v>0.03677409985101048</v>
+        <v>0.03677496638652267</v>
       </c>
     </row>
     <row r="3">
@@ -824,40 +824,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02705031270108093</v>
+        <v>0.02705080294781807</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03228255425366702</v>
+        <v>0.03228316328064779</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03078926637774642</v>
+        <v>0.03079036078286011</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0005147233710181068</v>
+        <v>0.0005149071033118289</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0009245265702002489</v>
+        <v>-0.0009244270615855942</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.749536005062632e-05</v>
+        <v>-2.728254732659065e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>0.004815778593322297</v>
+        <v>0.004815543301096934</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02432640440575425</v>
+        <v>0.02432564935901551</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01423486301403834</v>
+        <v>0.0142382150474984</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0282690508669</v>
+        <v>0.02827016696506105</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.006924106176672476</v>
+        <v>-0.00692370383767239</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04051413872263669</v>
+        <v>0.04051507449457625</v>
       </c>
     </row>
     <row r="4">
@@ -867,40 +867,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02717108089842512</v>
+        <v>0.02717185745198413</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03078926637774642</v>
+        <v>0.03079036078286011</v>
       </c>
       <c r="D4" t="n">
-        <v>0.04096377209129554</v>
+        <v>0.04096495714434405</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004490356898721208</v>
+        <v>0.0004493485049194264</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0009772348987412891</v>
+        <v>-0.0009771356352856579</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.092347514908783e-05</v>
+        <v>-1.040834127042788e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00598284375047626</v>
+        <v>0.005981501273544076</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02347948778986474</v>
+        <v>0.02347719005804366</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01601750702113731</v>
+        <v>0.01602894972525363</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0298813022857886</v>
+        <v>0.02988257543607003</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007009201483147245</v>
+        <v>-0.007008099780740143</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04655339091380395</v>
+        <v>0.04655601989557639</v>
       </c>
     </row>
     <row r="5">
@@ -910,40 +910,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.000333396862655863</v>
+        <v>0.0003335598448687919</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005147233710181068</v>
+        <v>0.0005149071033118289</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0004490356898721208</v>
+        <v>0.0004493485049194264</v>
       </c>
       <c r="E5" t="n">
-        <v>0.00254370286938505</v>
+        <v>0.002543746417014282</v>
       </c>
       <c r="F5" t="n">
-        <v>0.00148218237588971</v>
+        <v>0.001482213485943721</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002042228304807083</v>
+        <v>0.002042293721779925</v>
       </c>
       <c r="H5" t="n">
-        <v>0.002269208916107364</v>
+        <v>0.002269146952458502</v>
       </c>
       <c r="I5" t="n">
-        <v>0.002079815580105561</v>
+        <v>0.002079680642583018</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.0007008118460263069</v>
+        <v>-0.0006999222453762505</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0004803369407737381</v>
+        <v>0.0004806858392307718</v>
       </c>
       <c r="L5" t="n">
-        <v>0.005761292209264112</v>
+        <v>0.005761392331357792</v>
       </c>
       <c r="M5" t="n">
-        <v>3.994710976774526e-05</v>
+        <v>4.019914575474695e-05</v>
       </c>
     </row>
     <row r="6">
@@ -953,40 +953,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.001189442191261068</v>
+        <v>-0.001189382735895836</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.0009245265702002489</v>
+        <v>-0.0009244270615855942</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0009772348987412891</v>
+        <v>-0.0009771356352856579</v>
       </c>
       <c r="E6" t="n">
-        <v>0.00148218237588971</v>
+        <v>0.001482213485943721</v>
       </c>
       <c r="F6" t="n">
-        <v>0.001536449860786993</v>
+        <v>0.001536456953108964</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001572305482666053</v>
+        <v>0.001572361806140079</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00186845068242548</v>
+        <v>0.001868352461331721</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0003559723338068283</v>
+        <v>0.0003557929715395232</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.001185230637683308</v>
+        <v>-0.001184262318568055</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.001106653588632952</v>
+        <v>-0.001106555146895892</v>
       </c>
       <c r="L6" t="n">
-        <v>0.004361708697666991</v>
+        <v>0.004361828556489756</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.001505339436466972</v>
+        <v>-0.001505080403863565</v>
       </c>
     </row>
     <row r="7">
@@ -996,40 +996,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.000384462676792857</v>
+        <v>-0.0003842762657988831</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.749536005062632e-05</v>
+        <v>-2.728254732659065e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.092347514908783e-05</v>
+        <v>-1.040834127042788e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002042228304807083</v>
+        <v>0.002042293721779925</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001572305482666053</v>
+        <v>0.001572361806140079</v>
       </c>
       <c r="G7" t="n">
-        <v>0.003392818703741044</v>
+        <v>0.003392886125444758</v>
       </c>
       <c r="H7" t="n">
-        <v>0.003051702675547901</v>
+        <v>0.00305169025955567</v>
       </c>
       <c r="I7" t="n">
-        <v>0.00139464176020171</v>
+        <v>0.00139438535800788</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0009338399556922046</v>
+        <v>0.000934686581671446</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.0002782008106463274</v>
+        <v>-0.0002776690956172005</v>
       </c>
       <c r="L7" t="n">
-        <v>0.006216564708259299</v>
+        <v>0.006216702681890844</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001211401917078383</v>
+        <v>0.0001214006490508785</v>
       </c>
     </row>
     <row r="8">
@@ -1039,40 +1039,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001567662776933946</v>
+        <v>0.00156736672673012</v>
       </c>
       <c r="C8" t="n">
-        <v>0.004815778593322297</v>
+        <v>0.004815543301096934</v>
       </c>
       <c r="D8" t="n">
-        <v>0.00598284375047626</v>
+        <v>0.005981501273544076</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002269208916107364</v>
+        <v>0.002269146952458502</v>
       </c>
       <c r="F8" t="n">
-        <v>0.00186845068242548</v>
+        <v>0.001868352461331721</v>
       </c>
       <c r="G8" t="n">
-        <v>0.003051702675547901</v>
+        <v>0.00305169025955567</v>
       </c>
       <c r="H8" t="n">
-        <v>0.02727611014739878</v>
+        <v>0.02727530884525452</v>
       </c>
       <c r="I8" t="n">
-        <v>0.003576973333025768</v>
+        <v>0.003576499988979515</v>
       </c>
       <c r="J8" t="n">
-        <v>0.007495680830096611</v>
+        <v>0.007499557165991863</v>
       </c>
       <c r="K8" t="n">
-        <v>0.001883252046567955</v>
+        <v>0.001881980740895433</v>
       </c>
       <c r="L8" t="n">
-        <v>0.005267248349672161</v>
+        <v>0.005267438197806618</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01259414405596525</v>
+        <v>0.01259465646187742</v>
       </c>
     </row>
     <row r="9">
@@ -1082,40 +1082,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02590033361957083</v>
+        <v>0.0258995946128974</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02432640440575425</v>
+        <v>0.02432564935901551</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02347948778986474</v>
+        <v>0.02347719005804366</v>
       </c>
       <c r="E9" t="n">
-        <v>0.002079815580105561</v>
+        <v>0.002079680642583018</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003559723338068283</v>
+        <v>0.0003557929715395232</v>
       </c>
       <c r="G9" t="n">
-        <v>0.00139464176020171</v>
+        <v>0.00139438535800788</v>
       </c>
       <c r="H9" t="n">
-        <v>0.003576973333025768</v>
+        <v>0.003576499988979515</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03953331932102008</v>
+        <v>0.03953366644051844</v>
       </c>
       <c r="J9" t="n">
-        <v>0.009741445968415129</v>
+        <v>0.009741694011178076</v>
       </c>
       <c r="K9" t="n">
-        <v>0.02463516539174786</v>
+        <v>0.02463289092062435</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.001700509511680643</v>
+        <v>-0.001700760174598437</v>
       </c>
       <c r="M9" t="n">
-        <v>0.03105413838978375</v>
+        <v>0.03105369104893073</v>
       </c>
     </row>
     <row r="10">
@@ -1125,40 +1125,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.01298417150365833</v>
+        <v>0.01298748098504069</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01423486301403834</v>
+        <v>0.0142382150474984</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01601750702113731</v>
+        <v>0.01602894972525363</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0007008118460263069</v>
+        <v>-0.0006999222453762505</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.001185230637683308</v>
+        <v>-0.001184262318568055</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0009338399556922046</v>
+        <v>0.000934686581671446</v>
       </c>
       <c r="H10" t="n">
-        <v>0.007495680830096611</v>
+        <v>0.007499557165991863</v>
       </c>
       <c r="I10" t="n">
-        <v>0.009741445968415129</v>
+        <v>0.009741694011178076</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0446006486456187</v>
+        <v>0.04458887589908082</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01189300389162079</v>
+        <v>0.01190416654130541</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.006830686291870362</v>
+        <v>-0.006830394607750457</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02548618581130556</v>
+        <v>0.02548627555122637</v>
       </c>
     </row>
     <row r="11">
@@ -1168,40 +1168,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.03339183273804214</v>
+        <v>0.03339260737938018</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0282690508669</v>
+        <v>0.02827016696506105</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0298813022857886</v>
+        <v>0.02988257543607003</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0004803369407737381</v>
+        <v>0.0004806858392307718</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.001106653588632952</v>
+        <v>-0.001106555146895892</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0002782008106463274</v>
+        <v>-0.0002776690956172005</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001883252046567955</v>
+        <v>0.001881980740895433</v>
       </c>
       <c r="I11" t="n">
-        <v>0.02463516539174786</v>
+        <v>0.02463289092062435</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01189300389162079</v>
+        <v>0.01190416654130541</v>
       </c>
       <c r="K11" t="n">
-        <v>0.04274739260848172</v>
+        <v>0.04274868014403798</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.006334950366969848</v>
+        <v>-0.006333880878105161</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03972757972848921</v>
+        <v>0.03973016885097099</v>
       </c>
     </row>
     <row r="12">
@@ -1211,40 +1211,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.006985008289441838</v>
+        <v>-0.006984655662240311</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.006924106176672476</v>
+        <v>-0.00692370383767239</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.007009201483147245</v>
+        <v>-0.007008099780740143</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005761292209264112</v>
+        <v>0.005761392331357792</v>
       </c>
       <c r="F12" t="n">
-        <v>0.004361708697666991</v>
+        <v>0.004361828556489756</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006216564708259299</v>
+        <v>0.006216702681890844</v>
       </c>
       <c r="H12" t="n">
-        <v>0.005267248349672161</v>
+        <v>0.005267438197806618</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.001700509511680643</v>
+        <v>-0.001700760174598437</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.006830686291870362</v>
+        <v>-0.006830394607750457</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.006334950366969848</v>
+        <v>-0.006333880878105161</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0223760349350659</v>
+        <v>0.02237615003679361</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.01025788740331246</v>
+        <v>-0.0102576124092389</v>
       </c>
     </row>
     <row r="13">
@@ -1254,40 +1254,40 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.03677409985101048</v>
+        <v>0.03677496638652267</v>
       </c>
       <c r="C13" t="n">
-        <v>0.04051413872263669</v>
+        <v>0.04051507449457625</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04655339091380395</v>
+        <v>0.04655601989557639</v>
       </c>
       <c r="E13" t="n">
-        <v>3.994710976774526e-05</v>
+        <v>4.019914575474695e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.001505339436466972</v>
+        <v>-0.001505080403863565</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0001211401917078383</v>
+        <v>0.0001214006490508785</v>
       </c>
       <c r="H13" t="n">
-        <v>0.01259414405596525</v>
+        <v>0.01259465646187742</v>
       </c>
       <c r="I13" t="n">
-        <v>0.03105413838978375</v>
+        <v>0.03105369104893073</v>
       </c>
       <c r="J13" t="n">
-        <v>0.02548618581130556</v>
+        <v>0.02548627555122637</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03972757972848921</v>
+        <v>0.03973016885097099</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.01025788740331246</v>
+        <v>-0.0102576124092389</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1179567242533223</v>
+        <v>0.1179573451049781</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix portfolio audit correctness and handoff docs
</commit_message>
<xml_diff>
--- a/reports/excel/optimized_portfolios.xlsx
+++ b/reports/excel/optimized_portfolios.xlsx
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5000000000000009</v>
+        <v>0.4999999999999969</v>
       </c>
     </row>
     <row r="3">
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05000000000000073</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="4">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1499999999999996</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1499999999999997</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="12">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1499999999999997</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="13">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1358956347461182</v>
+        <v>0.1358956629588761</v>
       </c>
     </row>
     <row r="3">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0739750553109757</v>
+        <v>0.07397505531097548</v>
       </c>
     </row>
     <row r="4">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04133315844834007</v>
+        <v>0.0413331788988891</v>
       </c>
     </row>
     <row r="5">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0236045698975873</v>
+        <v>0.02360459461273678</v>
       </c>
     </row>
     <row r="6">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01934128567286342</v>
+        <v>0.01934125118458563</v>
       </c>
     </row>
     <row r="7">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.07645137401388813</v>
+        <v>0.0764513913967344</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1869328080968509</v>
+        <v>0.1869328019787047</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.02352762072477277</v>
+        <v>0.02352761231407663</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.04413709254914255</v>
+        <v>-0.04413708768693014</v>
       </c>
     </row>
   </sheetData>
@@ -781,40 +781,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03061090257805427</v>
+        <v>0.03061089887725833</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02705080294781807</v>
+        <v>0.02705081401796674</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02717185745198413</v>
+        <v>0.02717187229149563</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003335598448687919</v>
+        <v>0.0003335130338385384</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.001189382735895836</v>
+        <v>-0.001189368518419001</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0003842762657988831</v>
+        <v>-0.0003842548733471857</v>
       </c>
       <c r="H2" t="n">
-        <v>0.00156736672673012</v>
+        <v>0.001567361397464201</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0258995946128974</v>
+        <v>0.02589959187006571</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01298748098504069</v>
+        <v>0.012987473031258</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03339260737938018</v>
+        <v>0.03339262528299671</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006984655662240311</v>
+        <v>-0.006984621003437382</v>
       </c>
       <c r="M2" t="n">
-        <v>0.03677496638652267</v>
+        <v>0.03677497801047156</v>
       </c>
     </row>
     <row r="3">
@@ -824,40 +824,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02705080294781807</v>
+        <v>0.02705081401796674</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03228316328064779</v>
+        <v>0.03228313934186632</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03079036078286011</v>
+        <v>0.03079035115291501</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0005149071033118289</v>
+        <v>0.0005148724702480656</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0009244270615855942</v>
+        <v>-0.0009244284540890877</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.728254732659065e-05</v>
+        <v>-2.725673034116413e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>0.004815543301096934</v>
+        <v>0.004815526920974634</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02432564935901551</v>
+        <v>0.02432562360171144</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0142382150474984</v>
+        <v>0.0142381999698698</v>
       </c>
       <c r="K3" t="n">
-        <v>0.02827016696506105</v>
+        <v>0.0282701811365884</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.00692370383767239</v>
+        <v>-0.006923667280574777</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04051507449457625</v>
+        <v>0.0405150600431775</v>
       </c>
     </row>
     <row r="4">
@@ -867,40 +867,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02717185745198413</v>
+        <v>0.02717187229149563</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03079036078286011</v>
+        <v>0.03079035115291501</v>
       </c>
       <c r="D4" t="n">
-        <v>0.04096495714434405</v>
+        <v>0.04096497851722791</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004493485049194264</v>
+        <v>0.0004493102715919113</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0009771356352856579</v>
+        <v>-0.000977144317954698</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.040834127042788e-05</v>
+        <v>-1.038391225905761e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.005981501273544076</v>
+        <v>0.005981506360719041</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02347719005804366</v>
+        <v>0.02347715793356256</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01602894972525363</v>
+        <v>0.01602897102982188</v>
       </c>
       <c r="K4" t="n">
-        <v>0.02988257543607003</v>
+        <v>0.02988258708009146</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007008099780740143</v>
+        <v>-0.007008065318509722</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04655601989557639</v>
+        <v>0.04655602563398361</v>
       </c>
     </row>
     <row r="5">
@@ -910,40 +910,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0003335598448687919</v>
+        <v>0.0003335130338385384</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005149071033118289</v>
+        <v>0.0005148724702480656</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0004493485049194264</v>
+        <v>0.0004493102715919113</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002543746417014282</v>
+        <v>0.002543744061922126</v>
       </c>
       <c r="F5" t="n">
-        <v>0.001482213485943721</v>
+        <v>0.001482215243773234</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002042293721779925</v>
+        <v>0.002042296691445654</v>
       </c>
       <c r="H5" t="n">
-        <v>0.002269146952458502</v>
+        <v>0.002269140971893195</v>
       </c>
       <c r="I5" t="n">
-        <v>0.002079680642583018</v>
+        <v>0.002079609540341389</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.0006999222453762505</v>
+        <v>-0.0006999370668423981</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0004806858392307718</v>
+        <v>0.0004806419711097897</v>
       </c>
       <c r="L5" t="n">
-        <v>0.005761392331357792</v>
+        <v>0.005761418208239361</v>
       </c>
       <c r="M5" t="n">
-        <v>4.019914575474695e-05</v>
+        <v>4.01545383205874e-05</v>
       </c>
     </row>
     <row r="6">
@@ -953,40 +953,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.001189382735895836</v>
+        <v>-0.001189368518419001</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.0009244270615855942</v>
+        <v>-0.0009244284540890877</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0009771356352856579</v>
+        <v>-0.000977144317954698</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001482213485943721</v>
+        <v>0.001482215243773234</v>
       </c>
       <c r="F6" t="n">
-        <v>0.001536456953108964</v>
+        <v>0.001536448234343431</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001572361806140079</v>
+        <v>0.001572354591926645</v>
       </c>
       <c r="H6" t="n">
-        <v>0.001868352461331721</v>
+        <v>0.001868354111390807</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0003557929715395232</v>
+        <v>0.0003557765070196019</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.001184262318568055</v>
+        <v>-0.001184252333746811</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.001106555146895892</v>
+        <v>-0.001106532526188704</v>
       </c>
       <c r="L6" t="n">
-        <v>0.004361828556489756</v>
+        <v>0.004361813229243917</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.001505080403863565</v>
+        <v>-0.001505101642085883</v>
       </c>
     </row>
     <row r="7">
@@ -996,40 +996,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0003842762657988831</v>
+        <v>-0.0003842548733471857</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.728254732659065e-05</v>
+        <v>-2.725673034116413e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.040834127042788e-05</v>
+        <v>-1.038391225905761e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002042293721779925</v>
+        <v>0.002042296691445654</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001572361806140079</v>
+        <v>0.001572354591926645</v>
       </c>
       <c r="G7" t="n">
-        <v>0.003392886125444758</v>
+        <v>0.003392882283836251</v>
       </c>
       <c r="H7" t="n">
-        <v>0.00305169025955567</v>
+        <v>0.003051673619136453</v>
       </c>
       <c r="I7" t="n">
-        <v>0.00139438535800788</v>
+        <v>0.001394411734970172</v>
       </c>
       <c r="J7" t="n">
-        <v>0.000934686581671446</v>
+        <v>0.0009346733517646667</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.0002776690956172005</v>
+        <v>-0.000277655604992854</v>
       </c>
       <c r="L7" t="n">
-        <v>0.006216702681890844</v>
+        <v>0.006216693068717635</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001214006490508785</v>
+        <v>0.0001214325333986389</v>
       </c>
     </row>
     <row r="8">
@@ -1039,40 +1039,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.00156736672673012</v>
+        <v>0.001567361397464201</v>
       </c>
       <c r="C8" t="n">
-        <v>0.004815543301096934</v>
+        <v>0.004815526920974634</v>
       </c>
       <c r="D8" t="n">
-        <v>0.005981501273544076</v>
+        <v>0.005981506360719041</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002269146952458502</v>
+        <v>0.002269140971893195</v>
       </c>
       <c r="F8" t="n">
-        <v>0.001868352461331721</v>
+        <v>0.001868354111390807</v>
       </c>
       <c r="G8" t="n">
-        <v>0.00305169025955567</v>
+        <v>0.003051673619136453</v>
       </c>
       <c r="H8" t="n">
-        <v>0.02727530884525452</v>
+        <v>0.02727530881726122</v>
       </c>
       <c r="I8" t="n">
-        <v>0.003576499988979515</v>
+        <v>0.003576483152335444</v>
       </c>
       <c r="J8" t="n">
-        <v>0.007499557165991863</v>
+        <v>0.007499557188386178</v>
       </c>
       <c r="K8" t="n">
-        <v>0.001881980740895433</v>
+        <v>0.00188196977676326</v>
       </c>
       <c r="L8" t="n">
-        <v>0.005267438197806618</v>
+        <v>0.005267438323969596</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01259465646187742</v>
+        <v>0.01259465894192016</v>
       </c>
     </row>
     <row r="9">
@@ -1082,40 +1082,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0258995946128974</v>
+        <v>0.02589959187006571</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02432564935901551</v>
+        <v>0.02432562360171144</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02347719005804366</v>
+        <v>0.02347715793356256</v>
       </c>
       <c r="E9" t="n">
-        <v>0.002079680642583018</v>
+        <v>0.002079609540341389</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003557929715395232</v>
+        <v>0.0003557765070196019</v>
       </c>
       <c r="G9" t="n">
-        <v>0.00139438535800788</v>
+        <v>0.001394411734970172</v>
       </c>
       <c r="H9" t="n">
-        <v>0.003576499988979515</v>
+        <v>0.003576483152335444</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03953366644051844</v>
+        <v>0.03953362211180587</v>
       </c>
       <c r="J9" t="n">
-        <v>0.009741694011178076</v>
+        <v>0.009741664693250383</v>
       </c>
       <c r="K9" t="n">
-        <v>0.02463289092062435</v>
+        <v>0.02463289384379418</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.001700760174598437</v>
+        <v>-0.00170069631242235</v>
       </c>
       <c r="M9" t="n">
-        <v>0.03105369104893073</v>
+        <v>0.03105365196145685</v>
       </c>
     </row>
     <row r="10">
@@ -1125,40 +1125,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.01298748098504069</v>
+        <v>0.012987473031258</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0142382150474984</v>
+        <v>0.0142381999698698</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01602894972525363</v>
+        <v>0.01602897102982188</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0006999222453762505</v>
+        <v>-0.0006999370668423981</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.001184262318568055</v>
+        <v>-0.001184252333746811</v>
       </c>
       <c r="G10" t="n">
-        <v>0.000934686581671446</v>
+        <v>0.0009346733517646667</v>
       </c>
       <c r="H10" t="n">
-        <v>0.007499557165991863</v>
+        <v>0.007499557188386178</v>
       </c>
       <c r="I10" t="n">
-        <v>0.009741694011178076</v>
+        <v>0.009741664693250383</v>
       </c>
       <c r="J10" t="n">
-        <v>0.04458887589908082</v>
+        <v>0.0445888759227873</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01190416654130541</v>
+        <v>0.0119041974920161</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.006830394607750457</v>
+        <v>-0.006830406752205046</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02548627555122637</v>
+        <v>0.02548627036454772</v>
       </c>
     </row>
     <row r="11">
@@ -1168,40 +1168,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.03339260737938018</v>
+        <v>0.03339262528299671</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02827016696506105</v>
+        <v>0.0282701811365884</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02988257543607003</v>
+        <v>0.02988258708009146</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0004806858392307718</v>
+        <v>0.0004806419711097897</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.001106555146895892</v>
+        <v>-0.001106532526188704</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0002776690956172005</v>
+        <v>-0.000277655604992854</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001881980740895433</v>
+        <v>0.00188196977676326</v>
       </c>
       <c r="I11" t="n">
-        <v>0.02463289092062435</v>
+        <v>0.02463289384379418</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01190416654130541</v>
+        <v>0.0119041974920161</v>
       </c>
       <c r="K11" t="n">
-        <v>0.04274868014403798</v>
+        <v>0.04274873465801343</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.006333880878105161</v>
+        <v>-0.006333847877437349</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03973016885097099</v>
+        <v>0.03973017197635876</v>
       </c>
     </row>
     <row r="12">
@@ -1211,40 +1211,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.006984655662240311</v>
+        <v>-0.006984621003437382</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.00692370383767239</v>
+        <v>-0.006923667280574777</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.007008099780740143</v>
+        <v>-0.007008065318509722</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005761392331357792</v>
+        <v>0.005761418208239361</v>
       </c>
       <c r="F12" t="n">
-        <v>0.004361828556489756</v>
+        <v>0.004361813229243917</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006216702681890844</v>
+        <v>0.006216693068717635</v>
       </c>
       <c r="H12" t="n">
-        <v>0.005267438197806618</v>
+        <v>0.005267438323969596</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.001700760174598437</v>
+        <v>-0.00170069631242235</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.006830394607750457</v>
+        <v>-0.006830406752205046</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.006333880878105161</v>
+        <v>-0.006333847877437349</v>
       </c>
       <c r="L12" t="n">
-        <v>0.02237615003679361</v>
+        <v>0.0223761756207445</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.0102576124092389</v>
+        <v>-0.010257546193118</v>
       </c>
     </row>
     <row r="13">
@@ -1254,40 +1254,40 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.03677496638652267</v>
+        <v>0.03677497801047156</v>
       </c>
       <c r="C13" t="n">
-        <v>0.04051507449457625</v>
+        <v>0.0405150600431775</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04655601989557639</v>
+        <v>0.04655602563398361</v>
       </c>
       <c r="E13" t="n">
-        <v>4.019914575474695e-05</v>
+        <v>4.01545383205874e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.001505080403863565</v>
+        <v>-0.001505101642085883</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0001214006490508785</v>
+        <v>0.0001214325333986389</v>
       </c>
       <c r="H13" t="n">
-        <v>0.01259465646187742</v>
+        <v>0.01259465894192016</v>
       </c>
       <c r="I13" t="n">
-        <v>0.03105369104893073</v>
+        <v>0.03105365196145685</v>
       </c>
       <c r="J13" t="n">
-        <v>0.02548627555122637</v>
+        <v>0.02548627036454772</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03973016885097099</v>
+        <v>0.03973017197635876</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.0102576124092389</v>
+        <v>-0.010257546193118</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1179573451049781</v>
+        <v>0.1179573118165548</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Harden metrics and handoff provenance
</commit_message>
<xml_diff>
--- a/reports/excel/optimized_portfolios.xlsx
+++ b/reports/excel/optimized_portfolios.xlsx
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4999999999999969</v>
+        <v>0.4999999999999996</v>
       </c>
     </row>
     <row r="3">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1358956629588761</v>
+        <v>0.1358956460312208</v>
       </c>
     </row>
     <row r="3">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07397505531097548</v>
+        <v>0.07397507287384641</v>
       </c>
     </row>
     <row r="4">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0413331788988891</v>
+        <v>0.04133317889888888</v>
       </c>
     </row>
     <row r="5">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02360459461273678</v>
+        <v>0.02360460944183096</v>
       </c>
     </row>
     <row r="6">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01934125118458563</v>
+        <v>0.01934126842872241</v>
       </c>
     </row>
     <row r="7">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02813492693711761</v>
+        <v>0.02813492693711717</v>
       </c>
     </row>
     <row r="8">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0764513913967344</v>
+        <v>0.07645137401388835</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1869328019787047</v>
+        <v>0.1869328080968509</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.02352761231407663</v>
+        <v>0.02352761231407752</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.04413708768693014</v>
+        <v>-0.04413709254914255</v>
       </c>
     </row>
   </sheetData>
@@ -781,40 +781,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03061089887725833</v>
+        <v>0.03061090930553277</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02705081401796674</v>
+        <v>0.0270507792991646</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02717187229149563</v>
+        <v>0.02717186209420616</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003335130338385384</v>
+        <v>0.0003335122066596742</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.001189368518419001</v>
+        <v>-0.001189390589902162</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0003842548733471857</v>
+        <v>-0.0003842594444605382</v>
       </c>
       <c r="H2" t="n">
-        <v>0.001567361397464201</v>
+        <v>0.001567357154893825</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02589959187006571</v>
+        <v>0.02589959134413049</v>
       </c>
       <c r="J2" t="n">
-        <v>0.012987473031258</v>
+        <v>0.01298748646007673</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03339262528299671</v>
+        <v>0.03339261776322583</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006984621003437382</v>
+        <v>-0.006984640593376044</v>
       </c>
       <c r="M2" t="n">
-        <v>0.03677497801047156</v>
+        <v>0.0367749810481198</v>
       </c>
     </row>
     <row r="3">
@@ -824,40 +824,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02705081401796674</v>
+        <v>0.0270507792991646</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03228313934186632</v>
+        <v>0.03228310674556684</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03079035115291501</v>
+        <v>0.03079032474631012</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0005148724702480656</v>
+        <v>0.0005148586837932621</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0009244284540890877</v>
+        <v>-0.0009244456325860299</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.725673034116413e-05</v>
+        <v>-2.72617669617405e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>0.004815526920974634</v>
+        <v>0.004815531840869619</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02432562360171144</v>
+        <v>0.02432561693347147</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0142381999698698</v>
+        <v>0.01423820620791117</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0282701811365884</v>
+        <v>0.02827013311332008</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.006923667280574777</v>
+        <v>-0.006923680377722761</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0405150600431775</v>
+        <v>0.04051502426516504</v>
       </c>
     </row>
     <row r="4">
@@ -867,40 +867,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02717187229149563</v>
+        <v>0.02717186209420616</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03079035115291501</v>
+        <v>0.03079032474631012</v>
       </c>
       <c r="D4" t="n">
-        <v>0.04096497851722791</v>
+        <v>0.04096492544877061</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004493102715919113</v>
+        <v>0.0004493170524719703</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.000977144317954698</v>
+        <v>-0.0009771559324601401</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.038391225905761e-05</v>
+        <v>-1.040917179074284e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.005981506360719041</v>
+        <v>0.005981512065232805</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02347715793356256</v>
+        <v>0.02347717150694388</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01602897102982188</v>
+        <v>0.01602895992586994</v>
       </c>
       <c r="K4" t="n">
-        <v>0.02988258708009146</v>
+        <v>0.02988256548421785</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007008065318509722</v>
+        <v>-0.007008102409836713</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04655602563398361</v>
+        <v>0.04655603766065686</v>
       </c>
     </row>
     <row r="5">
@@ -910,40 +910,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0003335130338385384</v>
+        <v>0.0003335122066596742</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005148724702480656</v>
+        <v>0.0005148586837932621</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0004493102715919113</v>
+        <v>0.0004493170524719703</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002543744061922126</v>
+        <v>0.002543742618225573</v>
       </c>
       <c r="F5" t="n">
-        <v>0.001482215243773234</v>
+        <v>0.001482213254900332</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002042296691445654</v>
+        <v>0.002042298187924367</v>
       </c>
       <c r="H5" t="n">
-        <v>0.002269140971893195</v>
+        <v>0.002269123573513316</v>
       </c>
       <c r="I5" t="n">
-        <v>0.002079609540341389</v>
+        <v>0.002079618132607971</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.0006999370668423981</v>
+        <v>-0.0006999624799380566</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0004806419711097897</v>
+        <v>0.0004806321856144807</v>
       </c>
       <c r="L5" t="n">
-        <v>0.005761418208239361</v>
+        <v>0.005761421904333723</v>
       </c>
       <c r="M5" t="n">
-        <v>4.01545383205874e-05</v>
+        <v>4.013457507717371e-05</v>
       </c>
     </row>
     <row r="6">
@@ -953,40 +953,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.001189368518419001</v>
+        <v>-0.001189390589902162</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.0009244284540890877</v>
+        <v>-0.0009244456325860299</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.000977144317954698</v>
+        <v>-0.0009771559324601401</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001482215243773234</v>
+        <v>0.001482213254900332</v>
       </c>
       <c r="F6" t="n">
-        <v>0.001536448234343431</v>
+        <v>0.001536443277855507</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001572354591926645</v>
+        <v>0.001572348034740214</v>
       </c>
       <c r="H6" t="n">
-        <v>0.001868354111390807</v>
+        <v>0.001868350619897444</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0003557765070196019</v>
+        <v>0.0003557520837447833</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.001184252333746811</v>
+        <v>-0.001184271512799413</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.001106532526188704</v>
+        <v>-0.001106553620412519</v>
       </c>
       <c r="L6" t="n">
-        <v>0.004361813229243917</v>
+        <v>0.004361808912499382</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.001505101642085883</v>
+        <v>-0.001505101411058717</v>
       </c>
     </row>
     <row r="7">
@@ -996,40 +996,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0003842548733471857</v>
+        <v>-0.0003842594444605382</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.725673034116413e-05</v>
+        <v>-2.72617669617405e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.038391225905761e-05</v>
+        <v>-1.040917179074284e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002042296691445654</v>
+        <v>0.002042298187924367</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001572354591926645</v>
+        <v>0.001572348034740214</v>
       </c>
       <c r="G7" t="n">
-        <v>0.003392882283836251</v>
+        <v>0.003392883856740153</v>
       </c>
       <c r="H7" t="n">
-        <v>0.003051673619136453</v>
+        <v>0.003051675643119465</v>
       </c>
       <c r="I7" t="n">
-        <v>0.001394411734970172</v>
+        <v>0.001394380513296612</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0009346733517646667</v>
+        <v>0.0009346933377429707</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.000277655604992854</v>
+        <v>-0.0002776521611665862</v>
       </c>
       <c r="L7" t="n">
-        <v>0.006216693068717635</v>
+        <v>0.006216691367162084</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001214325333986389</v>
+        <v>0.000121415935983815</v>
       </c>
     </row>
     <row r="8">
@@ -1039,40 +1039,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001567361397464201</v>
+        <v>0.001567357154893825</v>
       </c>
       <c r="C8" t="n">
-        <v>0.004815526920974634</v>
+        <v>0.004815531840869619</v>
       </c>
       <c r="D8" t="n">
-        <v>0.005981506360719041</v>
+        <v>0.005981512065232805</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002269140971893195</v>
+        <v>0.002269123573513316</v>
       </c>
       <c r="F8" t="n">
-        <v>0.001868354111390807</v>
+        <v>0.001868350619897444</v>
       </c>
       <c r="G8" t="n">
-        <v>0.003051673619136453</v>
+        <v>0.003051675643119465</v>
       </c>
       <c r="H8" t="n">
-        <v>0.02727530881726122</v>
+        <v>0.02727530884290736</v>
       </c>
       <c r="I8" t="n">
-        <v>0.003576483152335444</v>
+        <v>0.003576501039437429</v>
       </c>
       <c r="J8" t="n">
-        <v>0.007499557188386178</v>
+        <v>0.007499557143196277</v>
       </c>
       <c r="K8" t="n">
-        <v>0.00188196977676326</v>
+        <v>0.001881975010981764</v>
       </c>
       <c r="L8" t="n">
-        <v>0.005267438323969596</v>
+        <v>0.005267417930384048</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01259465894192016</v>
+        <v>0.0125946490610357</v>
       </c>
     </row>
     <row r="9">
@@ -1082,40 +1082,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02589959187006571</v>
+        <v>0.02589959134413049</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02432562360171144</v>
+        <v>0.02432561693347147</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02347715793356256</v>
+        <v>0.02347717150694388</v>
       </c>
       <c r="E9" t="n">
-        <v>0.002079609540341389</v>
+        <v>0.002079618132607971</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003557765070196019</v>
+        <v>0.0003557520837447833</v>
       </c>
       <c r="G9" t="n">
-        <v>0.001394411734970172</v>
+        <v>0.001394380513296612</v>
       </c>
       <c r="H9" t="n">
-        <v>0.003576483152335444</v>
+        <v>0.003576501039437429</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03953362211180587</v>
+        <v>0.03953367723139406</v>
       </c>
       <c r="J9" t="n">
-        <v>0.009741664693250383</v>
+        <v>0.009741675005971739</v>
       </c>
       <c r="K9" t="n">
-        <v>0.02463289384379418</v>
+        <v>0.02463289412627353</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.00170069631242235</v>
+        <v>-0.001700725698457307</v>
       </c>
       <c r="M9" t="n">
-        <v>0.03105365196145685</v>
+        <v>0.03105369261513037</v>
       </c>
     </row>
     <row r="10">
@@ -1125,40 +1125,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.012987473031258</v>
+        <v>0.01298748646007673</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0142381999698698</v>
+        <v>0.01423820620791117</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01602897102982188</v>
+        <v>0.01602895992586994</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0006999370668423981</v>
+        <v>-0.0006999624799380566</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.001184252333746811</v>
+        <v>-0.001184271512799413</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0009346733517646667</v>
+        <v>0.0009346933377429707</v>
       </c>
       <c r="H10" t="n">
-        <v>0.007499557188386178</v>
+        <v>0.007499557143196277</v>
       </c>
       <c r="I10" t="n">
-        <v>0.009741664693250383</v>
+        <v>0.009741675005971739</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0445888759227873</v>
+        <v>0.0445888758441075</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0119041974920161</v>
+        <v>0.01190420287768578</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.006830406752205046</v>
+        <v>-0.006830389556282741</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02548627036454772</v>
+        <v>0.02548626408080827</v>
       </c>
     </row>
     <row r="11">
@@ -1168,40 +1168,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.03339262528299671</v>
+        <v>0.03339261776322583</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0282701811365884</v>
+        <v>0.02827013311332008</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02988258708009146</v>
+        <v>0.02988256548421785</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0004806419711097897</v>
+        <v>0.0004806321856144807</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.001106532526188704</v>
+        <v>-0.001106553620412519</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.000277655604992854</v>
+        <v>-0.0002776521611665862</v>
       </c>
       <c r="H11" t="n">
-        <v>0.00188196977676326</v>
+        <v>0.001881975010981764</v>
       </c>
       <c r="I11" t="n">
-        <v>0.02463289384379418</v>
+        <v>0.02463289412627353</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0119041974920161</v>
+        <v>0.01190420287768578</v>
       </c>
       <c r="K11" t="n">
-        <v>0.04274873465801343</v>
+        <v>0.04274869570773768</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.006333847877437349</v>
+        <v>-0.006333887495822869</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03973017197635876</v>
+        <v>0.03973016937793043</v>
       </c>
     </row>
     <row r="12">
@@ -1211,40 +1211,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.006984621003437382</v>
+        <v>-0.006984640593376044</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.006923667280574777</v>
+        <v>-0.006923680377722761</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.007008065318509722</v>
+        <v>-0.007008102409836713</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005761418208239361</v>
+        <v>0.005761421904333723</v>
       </c>
       <c r="F12" t="n">
-        <v>0.004361813229243917</v>
+        <v>0.004361808912499382</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006216693068717635</v>
+        <v>0.006216691367162084</v>
       </c>
       <c r="H12" t="n">
-        <v>0.005267438323969596</v>
+        <v>0.005267417930384048</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.00170069631242235</v>
+        <v>-0.001700725698457307</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.006830406752205046</v>
+        <v>-0.006830389556282741</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.006333847877437349</v>
+        <v>-0.006333887495822869</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0223761756207445</v>
+        <v>0.02237620329735396</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.010257546193118</v>
+        <v>-0.01025759340859155</v>
       </c>
     </row>
     <row r="13">
@@ -1254,40 +1254,40 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.03677497801047156</v>
+        <v>0.0367749810481198</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0405150600431775</v>
+        <v>0.04051502426516504</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04655602563398361</v>
+        <v>0.04655603766065686</v>
       </c>
       <c r="E13" t="n">
-        <v>4.01545383205874e-05</v>
+        <v>4.013457507717371e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.001505101642085883</v>
+        <v>-0.001505101411058717</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0001214325333986389</v>
+        <v>0.000121415935983815</v>
       </c>
       <c r="H13" t="n">
-        <v>0.01259465894192016</v>
+        <v>0.0125946490610357</v>
       </c>
       <c r="I13" t="n">
-        <v>0.03105365196145685</v>
+        <v>0.03105369261513037</v>
       </c>
       <c r="J13" t="n">
-        <v>0.02548627036454772</v>
+        <v>0.02548626408080827</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03973017197635876</v>
+        <v>0.03973016937793043</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.010257546193118</v>
+        <v>-0.01025759340859155</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1179573118165548</v>
+        <v>0.1179573176177185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update CI action pins
</commit_message>
<xml_diff>
--- a/reports/excel/optimized_portfolios.xlsx
+++ b/reports/excel/optimized_portfolios.xlsx
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4999999999999996</v>
+        <v>0.5000000000000028</v>
       </c>
     </row>
     <row r="3">
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000047</v>
       </c>
     </row>
     <row r="4">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.15</v>
+        <v>0.1499999999999986</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.15</v>
+        <v>0.1499999999999998</v>
       </c>
     </row>
     <row r="12">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1358956460312208</v>
+        <v>0.1358956516737717</v>
       </c>
     </row>
     <row r="3">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07397507287384641</v>
+        <v>0.07397507872813747</v>
       </c>
     </row>
     <row r="4">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04133317889888888</v>
+        <v>0.04133315844834007</v>
       </c>
     </row>
     <row r="5">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02360460944183096</v>
+        <v>0.02360452046731676</v>
       </c>
     </row>
     <row r="6">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01934126842872241</v>
+        <v>0.0193412741767689</v>
       </c>
     </row>
     <row r="7">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02813492693711717</v>
+        <v>0.02813493395493616</v>
       </c>
     </row>
     <row r="8">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.07645137401388835</v>
+        <v>0.07645136097675631</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1869328080968509</v>
+        <v>0.1869327958605598</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.02352761231407752</v>
+        <v>0.02352764595686629</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.04413709254914255</v>
+        <v>-0.044137092549142</v>
       </c>
     </row>
   </sheetData>
@@ -781,40 +781,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03061090930553277</v>
+        <v>0.03061091585168646</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0270507792991646</v>
+        <v>0.02705079674678561</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02717186209420616</v>
+        <v>0.02717187106467548</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003335122066596742</v>
+        <v>0.0003335046263432388</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.001189390589902162</v>
+        <v>-0.001189389848757407</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0003842594444605382</v>
+        <v>-0.0003842666882169936</v>
       </c>
       <c r="H2" t="n">
-        <v>0.001567357154893825</v>
+        <v>0.001567369876727225</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02589959134413049</v>
+        <v>0.02589960520281462</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01298748646007673</v>
+        <v>0.01298746710845889</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03339261776322583</v>
+        <v>0.03339262578189272</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006984640593376044</v>
+        <v>-0.006984632648182314</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0367749810481198</v>
+        <v>0.03677496618860314</v>
       </c>
     </row>
     <row r="3">
@@ -824,40 +824,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0270507792991646</v>
+        <v>0.02705079674678561</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03228310674556684</v>
+        <v>0.03228314363349966</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03079032474631012</v>
+        <v>0.03079037035853608</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0005148586837932621</v>
+        <v>0.0005148648251348672</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0009244456325860299</v>
+        <v>-0.0009244535926810831</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.72617669617405e-05</v>
+        <v>-2.726413228595986e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>0.004815531840869619</v>
+        <v>0.004815550005584293</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02432561693347147</v>
+        <v>0.02432564430783328</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01423820620791117</v>
+        <v>0.01423823592665975</v>
       </c>
       <c r="K3" t="n">
-        <v>0.02827013311332008</v>
+        <v>0.02827015146920691</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.006923680377722761</v>
+        <v>-0.006923672132899366</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04051502426516504</v>
+        <v>0.04051506590783106</v>
       </c>
     </row>
     <row r="4">
@@ -867,40 +867,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02717186209420616</v>
+        <v>0.02717187106467548</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03079032474631012</v>
+        <v>0.03079037035853608</v>
       </c>
       <c r="D4" t="n">
-        <v>0.04096492544877061</v>
+        <v>0.04096497225931768</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004493170524719703</v>
+        <v>0.0004493052426840275</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0009771559324601401</v>
+        <v>-0.0009771428749403982</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.040917179074284e-05</v>
+        <v>-1.040008783996816e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.005981512065232805</v>
+        <v>0.005981510438527741</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02347717150694388</v>
+        <v>0.02347718966925405</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01602895992586994</v>
+        <v>0.01602897692737991</v>
       </c>
       <c r="K4" t="n">
-        <v>0.02988256548421785</v>
+        <v>0.0298825686015476</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007008102409836713</v>
+        <v>-0.007008072402308412</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04655603766065686</v>
+        <v>0.04655603178803784</v>
       </c>
     </row>
     <row r="5">
@@ -910,40 +910,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0003335122066596742</v>
+        <v>0.0003335046263432388</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005148586837932621</v>
+        <v>0.0005148648251348672</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0004493170524719703</v>
+        <v>0.0004493052426840275</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002543742618225573</v>
+        <v>0.002543746448674608</v>
       </c>
       <c r="F5" t="n">
-        <v>0.001482213254900332</v>
+        <v>0.001482214340200439</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002042298187924367</v>
+        <v>0.002042302700719726</v>
       </c>
       <c r="H5" t="n">
-        <v>0.002269123573513316</v>
+        <v>0.002269127237661919</v>
       </c>
       <c r="I5" t="n">
-        <v>0.002079618132607971</v>
+        <v>0.002079619851561016</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.0006999624799380566</v>
+        <v>-0.0006999528313996019</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0004806321856144807</v>
+        <v>0.0004806151576768403</v>
       </c>
       <c r="L5" t="n">
-        <v>0.005761421904333723</v>
+        <v>0.00576142691507104</v>
       </c>
       <c r="M5" t="n">
-        <v>4.013457507717371e-05</v>
+        <v>4.016612443580877e-05</v>
       </c>
     </row>
     <row r="6">
@@ -953,40 +953,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.001189390589902162</v>
+        <v>-0.001189389848757407</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.0009244456325860299</v>
+        <v>-0.0009244535926810831</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0009771559324601401</v>
+        <v>-0.0009771428749403982</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001482213254900332</v>
+        <v>0.001482214340200439</v>
       </c>
       <c r="F6" t="n">
-        <v>0.001536443277855507</v>
+        <v>0.001536448398484986</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001572348034740214</v>
+        <v>0.001572355117201128</v>
       </c>
       <c r="H6" t="n">
-        <v>0.001868350619897444</v>
+        <v>0.001868354505684352</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0003557520837447833</v>
+        <v>0.0003557680516387176</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.001184271512799413</v>
+        <v>-0.001184252544507377</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.001106553620412519</v>
+        <v>-0.001106555693483212</v>
       </c>
       <c r="L6" t="n">
-        <v>0.004361808912499382</v>
+        <v>0.004361811919052664</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.001505101411058717</v>
+        <v>-0.001505117009196318</v>
       </c>
     </row>
     <row r="7">
@@ -996,40 +996,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0003842594444605382</v>
+        <v>-0.0003842666882169936</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.72617669617405e-05</v>
+        <v>-2.726413228595986e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.040917179074284e-05</v>
+        <v>-1.040008783996816e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002042298187924367</v>
+        <v>0.002042302700719726</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001572348034740214</v>
+        <v>0.001572355117201128</v>
       </c>
       <c r="G7" t="n">
-        <v>0.003392883856740153</v>
+        <v>0.00339289296685449</v>
       </c>
       <c r="H7" t="n">
-        <v>0.003051675643119465</v>
+        <v>0.003051674813377302</v>
       </c>
       <c r="I7" t="n">
-        <v>0.001394380513296612</v>
+        <v>0.001394399487789729</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0009346933377429707</v>
+        <v>0.0009346939442439454</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.0002776521611665862</v>
+        <v>-0.0002776740321931119</v>
       </c>
       <c r="L7" t="n">
-        <v>0.006216691367162084</v>
+        <v>0.006216706243753326</v>
       </c>
       <c r="M7" t="n">
-        <v>0.000121415935983815</v>
+        <v>0.0001213940806772489</v>
       </c>
     </row>
     <row r="8">
@@ -1039,40 +1039,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001567357154893825</v>
+        <v>0.001567369876727225</v>
       </c>
       <c r="C8" t="n">
-        <v>0.004815531840869619</v>
+        <v>0.004815550005584293</v>
       </c>
       <c r="D8" t="n">
-        <v>0.005981512065232805</v>
+        <v>0.005981510438527741</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002269123573513316</v>
+        <v>0.002269127237661919</v>
       </c>
       <c r="F8" t="n">
-        <v>0.001868350619897444</v>
+        <v>0.001868354505684352</v>
       </c>
       <c r="G8" t="n">
-        <v>0.003051675643119465</v>
+        <v>0.003051674813377302</v>
       </c>
       <c r="H8" t="n">
-        <v>0.02727530884290736</v>
+        <v>0.02727530884825379</v>
       </c>
       <c r="I8" t="n">
-        <v>0.003576501039437429</v>
+        <v>0.003576497212273378</v>
       </c>
       <c r="J8" t="n">
-        <v>0.007499557143196277</v>
+        <v>0.00749955718718931</v>
       </c>
       <c r="K8" t="n">
-        <v>0.001881975010981764</v>
+        <v>0.001881980711318011</v>
       </c>
       <c r="L8" t="n">
-        <v>0.005267417930384048</v>
+        <v>0.005267436496113646</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0125946490610357</v>
+        <v>0.01259465896827418</v>
       </c>
     </row>
     <row r="9">
@@ -1082,40 +1082,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02589959134413049</v>
+        <v>0.02589960520281462</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02432561693347147</v>
+        <v>0.02432564430783328</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02347717150694388</v>
+        <v>0.02347718966925405</v>
       </c>
       <c r="E9" t="n">
-        <v>0.002079618132607971</v>
+        <v>0.002079619851561016</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003557520837447833</v>
+        <v>0.0003557680516387176</v>
       </c>
       <c r="G9" t="n">
-        <v>0.001394380513296612</v>
+        <v>0.001394399487789729</v>
       </c>
       <c r="H9" t="n">
-        <v>0.003576501039437429</v>
+        <v>0.003576497212273378</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03953367723139406</v>
+        <v>0.03953368134345276</v>
       </c>
       <c r="J9" t="n">
-        <v>0.009741675005971739</v>
+        <v>0.00974168648198012</v>
       </c>
       <c r="K9" t="n">
-        <v>0.02463289412627353</v>
+        <v>0.0246329029619418</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.001700725698457307</v>
+        <v>-0.001700713036666564</v>
       </c>
       <c r="M9" t="n">
-        <v>0.03105369261513037</v>
+        <v>0.0310536900294825</v>
       </c>
     </row>
     <row r="10">
@@ -1125,40 +1125,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.01298748646007673</v>
+        <v>0.01298746710845889</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01423820620791117</v>
+        <v>0.01423823592665975</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01602895992586994</v>
+        <v>0.01602897692737991</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0006999624799380566</v>
+        <v>-0.0006999528313996019</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.001184271512799413</v>
+        <v>-0.001184252544507377</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0009346933377429707</v>
+        <v>0.0009346939442439454</v>
       </c>
       <c r="H10" t="n">
-        <v>0.007499557143196277</v>
+        <v>0.00749955718718931</v>
       </c>
       <c r="I10" t="n">
-        <v>0.009741675005971739</v>
+        <v>0.00974168648198012</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0445888758441075</v>
+        <v>0.04458887595101676</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01190420287768578</v>
+        <v>0.01190418081690332</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.006830389556282741</v>
+        <v>-0.006830362556027613</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02548626408080827</v>
+        <v>0.0254862592067964</v>
       </c>
     </row>
     <row r="11">
@@ -1168,40 +1168,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.03339261776322583</v>
+        <v>0.03339262578189272</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02827013311332008</v>
+        <v>0.02827015146920691</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02988256548421785</v>
+        <v>0.0298825686015476</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0004806321856144807</v>
+        <v>0.0004806151576768403</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.001106553620412519</v>
+        <v>-0.001106555693483212</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0002776521611665862</v>
+        <v>-0.0002776740321931119</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001881975010981764</v>
+        <v>0.001881980711318011</v>
       </c>
       <c r="I11" t="n">
-        <v>0.02463289412627353</v>
+        <v>0.0246329029619418</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01190420287768578</v>
+        <v>0.01190418081690332</v>
       </c>
       <c r="K11" t="n">
-        <v>0.04274869570773768</v>
+        <v>0.04274868897782444</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.006333887495822869</v>
+        <v>-0.006333867158072055</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03973016937793043</v>
+        <v>0.03973017892135465</v>
       </c>
     </row>
     <row r="12">
@@ -1211,40 +1211,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.006984640593376044</v>
+        <v>-0.006984632648182314</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.006923680377722761</v>
+        <v>-0.006923672132899366</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.007008102409836713</v>
+        <v>-0.007008072402308412</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005761421904333723</v>
+        <v>0.00576142691507104</v>
       </c>
       <c r="F12" t="n">
-        <v>0.004361808912499382</v>
+        <v>0.004361811919052664</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006216691367162084</v>
+        <v>0.006216706243753326</v>
       </c>
       <c r="H12" t="n">
-        <v>0.005267417930384048</v>
+        <v>0.005267436496113646</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.001700725698457307</v>
+        <v>-0.001700713036666564</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.006830389556282741</v>
+        <v>-0.006830362556027613</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.006333887495822869</v>
+        <v>-0.006333867158072055</v>
       </c>
       <c r="L12" t="n">
-        <v>0.02237620329735396</v>
+        <v>0.02237618985940767</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.01025759340859155</v>
+        <v>-0.01025756880625418</v>
       </c>
     </row>
     <row r="13">
@@ -1254,40 +1254,40 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0367749810481198</v>
+        <v>0.03677496618860314</v>
       </c>
       <c r="C13" t="n">
-        <v>0.04051502426516504</v>
+        <v>0.04051506590783106</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04655603766065686</v>
+        <v>0.04655603178803784</v>
       </c>
       <c r="E13" t="n">
-        <v>4.013457507717371e-05</v>
+        <v>4.016612443580877e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.001505101411058717</v>
+        <v>-0.001505117009196318</v>
       </c>
       <c r="G13" t="n">
-        <v>0.000121415935983815</v>
+        <v>0.0001213940806772489</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0125946490610357</v>
+        <v>0.01259465896827418</v>
       </c>
       <c r="I13" t="n">
-        <v>0.03105369261513037</v>
+        <v>0.0310536900294825</v>
       </c>
       <c r="J13" t="n">
-        <v>0.02548626408080827</v>
+        <v>0.0254862592067964</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03973016937793043</v>
+        <v>0.03973017892135465</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.01025759340859155</v>
+        <v>-0.01025756880625418</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1179573176177185</v>
+        <v>0.1179573219649314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix report layout and document config options
</commit_message>
<xml_diff>
--- a/reports/excel/optimized_portfolios.xlsx
+++ b/reports/excel/optimized_portfolios.xlsx
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5000000000000028</v>
+        <v>0.5000000000000004</v>
       </c>
     </row>
     <row r="3">
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05000000000000047</v>
+        <v>0.05000000000000059</v>
       </c>
     </row>
     <row r="4">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1499999999999986</v>
+        <v>0.1499999999999988</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1499999999999998</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="12">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.15</v>
+        <v>0.149999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1358956516737717</v>
+        <v>0.1358956573163244</v>
       </c>
     </row>
     <row r="3">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04133315844834007</v>
+        <v>0.04133318298900024</v>
       </c>
     </row>
     <row r="5">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02360452046731676</v>
+        <v>0.02360456495455776</v>
       </c>
     </row>
     <row r="6">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0193412741767689</v>
+        <v>0.01934127417676823</v>
       </c>
     </row>
     <row r="7">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02813493395493616</v>
+        <v>0.02813491991929951</v>
       </c>
     </row>
     <row r="8">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.07645136097675631</v>
+        <v>0.07645139139673418</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1869327958605598</v>
+        <v>0.1869327775061258</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.02352764595686629</v>
+        <v>0.0235276039033816</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.044137092549142</v>
+        <v>-0.04413709741135363</v>
       </c>
     </row>
   </sheetData>
@@ -781,40 +781,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03061091585168646</v>
+        <v>0.03061089492413566</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02705079674678561</v>
+        <v>0.02705078862784563</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02717187106467548</v>
+        <v>0.02717187221882332</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003335046263432388</v>
+        <v>0.0003335410928770784</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.001189389848757407</v>
+        <v>-0.001189391677687678</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0003842666882169936</v>
+        <v>-0.000384270123600682</v>
       </c>
       <c r="H2" t="n">
-        <v>0.001567369876727225</v>
+        <v>0.001567361253756204</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02589960520281462</v>
+        <v>0.02589960777695037</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01298746710845889</v>
+        <v>0.01298748461776834</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03339262578189272</v>
+        <v>0.03339258820560981</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006984632648182314</v>
+        <v>-0.006984614515524904</v>
       </c>
       <c r="M2" t="n">
-        <v>0.03677496618860314</v>
+        <v>0.03677495510865</v>
       </c>
     </row>
     <row r="3">
@@ -824,40 +824,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02705079674678561</v>
+        <v>0.02705078862784563</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03228314363349966</v>
+        <v>0.03228315741260494</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03079037035853608</v>
+        <v>0.03079037988157218</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0005148648251348672</v>
+        <v>0.0005148830947617778</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0009244535926810831</v>
+        <v>-0.000924454193921033</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.726413228595986e-05</v>
+        <v>-2.727087635139866e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>0.004815550005584293</v>
+        <v>0.00481553388832663</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02432564430783328</v>
+        <v>0.02432564597094725</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01423823592665975</v>
+        <v>0.01423823011892062</v>
       </c>
       <c r="K3" t="n">
-        <v>0.02827015146920691</v>
+        <v>0.02827013491248067</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.006923672132899366</v>
+        <v>-0.006923664159927042</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04051506590783106</v>
+        <v>0.04051506380915469</v>
       </c>
     </row>
     <row r="4">
@@ -867,40 +867,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02717187106467548</v>
+        <v>0.02717187221882332</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03079037035853608</v>
+        <v>0.03079037988157218</v>
       </c>
       <c r="D4" t="n">
-        <v>0.04096497225931768</v>
+        <v>0.04096502102189881</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004493052426840275</v>
+        <v>0.0004493179162474735</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0009771428749403982</v>
+        <v>-0.0009771598922292232</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.040008783996816e-05</v>
+        <v>-1.039694793583059e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.005981510438527741</v>
+        <v>0.005981511564015721</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02347718966925405</v>
+        <v>0.02347723426395641</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01602897692737991</v>
+        <v>0.01602897485897988</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0298825686015476</v>
+        <v>0.029882581141819</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007008072402308412</v>
+        <v>-0.007008057251556645</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04655603178803784</v>
+        <v>0.04655606142444107</v>
       </c>
     </row>
     <row r="5">
@@ -910,40 +910,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0003335046263432388</v>
+        <v>0.0003335410928770784</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005148648251348672</v>
+        <v>0.0005148830947617778</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0004493052426840275</v>
+        <v>0.0004493179162474735</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002543746448674608</v>
+        <v>0.002543737655661055</v>
       </c>
       <c r="F5" t="n">
-        <v>0.001482214340200439</v>
+        <v>0.001482217925615223</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002042302700719726</v>
+        <v>0.002042299177977453</v>
       </c>
       <c r="H5" t="n">
-        <v>0.002269127237661919</v>
+        <v>0.002269131071656717</v>
       </c>
       <c r="I5" t="n">
-        <v>0.002079619851561016</v>
+        <v>0.002079660754669346</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.0006999528313996019</v>
+        <v>-0.0006999734703914388</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0004806151576768403</v>
+        <v>0.0004806581162570173</v>
       </c>
       <c r="L5" t="n">
-        <v>0.00576142691507104</v>
+        <v>0.00576139837511575</v>
       </c>
       <c r="M5" t="n">
-        <v>4.016612443580877e-05</v>
+        <v>4.019200736346342e-05</v>
       </c>
     </row>
     <row r="6">
@@ -953,40 +953,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.001189389848757407</v>
+        <v>-0.001189391677687678</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.0009244535926810831</v>
+        <v>-0.000924454193921033</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0009771428749403982</v>
+        <v>-0.0009771598922292232</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001482214340200439</v>
+        <v>0.001482217925615223</v>
       </c>
       <c r="F6" t="n">
-        <v>0.001536448398484986</v>
+        <v>0.001536453092732921</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001572355117201128</v>
+        <v>0.00157236338541709</v>
       </c>
       <c r="H6" t="n">
-        <v>0.001868354505684352</v>
+        <v>0.001868348128230625</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0003557680516387176</v>
+        <v>0.0003557686195830369</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.001184252544507377</v>
+        <v>-0.001184268645380405</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.001106555693483212</v>
+        <v>-0.001106551972723699</v>
       </c>
       <c r="L6" t="n">
-        <v>0.004361811919052664</v>
+        <v>0.004361823878065251</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.001505117009196318</v>
+        <v>-0.001505125204721985</v>
       </c>
     </row>
     <row r="7">
@@ -996,40 +996,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0003842666882169936</v>
+        <v>-0.000384270123600682</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.726413228595986e-05</v>
+        <v>-2.727087635139866e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.040008783996816e-05</v>
+        <v>-1.039694793583059e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002042302700719726</v>
+        <v>0.002042299177977453</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001572355117201128</v>
+        <v>0.00157236338541709</v>
       </c>
       <c r="G7" t="n">
-        <v>0.00339289296685449</v>
+        <v>0.003392902402128282</v>
       </c>
       <c r="H7" t="n">
-        <v>0.003051674813377302</v>
+        <v>0.003051686513386223</v>
       </c>
       <c r="I7" t="n">
-        <v>0.001394399487789729</v>
+        <v>0.001394384258620015</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0009346939442439454</v>
+        <v>0.0009346717114202901</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.0002776740321931119</v>
+        <v>-0.0002776720455737413</v>
       </c>
       <c r="L7" t="n">
-        <v>0.006216706243753326</v>
+        <v>0.006216703894578712</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001213940806772489</v>
+        <v>0.0001214081698984464</v>
       </c>
     </row>
     <row r="8">
@@ -1039,40 +1039,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001567369876727225</v>
+        <v>0.001567361253756204</v>
       </c>
       <c r="C8" t="n">
-        <v>0.004815550005584293</v>
+        <v>0.00481553388832663</v>
       </c>
       <c r="D8" t="n">
-        <v>0.005981510438527741</v>
+        <v>0.005981511564015721</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002269127237661919</v>
+        <v>0.002269131071656717</v>
       </c>
       <c r="F8" t="n">
-        <v>0.001868354505684352</v>
+        <v>0.001868348128230625</v>
       </c>
       <c r="G8" t="n">
-        <v>0.003051674813377302</v>
+        <v>0.003051686513386223</v>
       </c>
       <c r="H8" t="n">
-        <v>0.02727530884825379</v>
+        <v>0.02727530884611568</v>
       </c>
       <c r="I8" t="n">
-        <v>0.003576497212273378</v>
+        <v>0.003576485847236712</v>
       </c>
       <c r="J8" t="n">
-        <v>0.00749955718718931</v>
+        <v>0.007499557176965373</v>
       </c>
       <c r="K8" t="n">
-        <v>0.001881980711318011</v>
+        <v>0.001881975708770497</v>
       </c>
       <c r="L8" t="n">
-        <v>0.005267436496113646</v>
+        <v>0.005267434459916362</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01259465896827418</v>
+        <v>0.0125946562048136</v>
       </c>
     </row>
     <row r="9">
@@ -1082,40 +1082,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02589960520281462</v>
+        <v>0.02589960777695037</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02432564430783328</v>
+        <v>0.02432564597094725</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02347718966925405</v>
+        <v>0.02347723426395641</v>
       </c>
       <c r="E9" t="n">
-        <v>0.002079619851561016</v>
+        <v>0.002079660754669346</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003557680516387176</v>
+        <v>0.0003557686195830369</v>
       </c>
       <c r="G9" t="n">
-        <v>0.001394399487789729</v>
+        <v>0.001394384258620015</v>
       </c>
       <c r="H9" t="n">
-        <v>0.003576497212273378</v>
+        <v>0.003576485847236712</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03953368134345276</v>
+        <v>0.03953369135924182</v>
       </c>
       <c r="J9" t="n">
-        <v>0.00974168648198012</v>
+        <v>0.009741703143452796</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0246329029619418</v>
+        <v>0.02463290276657371</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.001700713036666564</v>
+        <v>-0.001700713853494101</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0310536900294825</v>
+        <v>0.03105372179720148</v>
       </c>
     </row>
     <row r="10">
@@ -1125,40 +1125,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.01298746710845889</v>
+        <v>0.01298748461776834</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01423823592665975</v>
+        <v>0.01423823011892062</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01602897692737991</v>
+        <v>0.01602897485897988</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0006999528313996019</v>
+        <v>-0.0006999734703914388</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.001184252544507377</v>
+        <v>-0.001184268645380405</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0009346939442439454</v>
+        <v>0.0009346717114202901</v>
       </c>
       <c r="H10" t="n">
-        <v>0.00749955718718931</v>
+        <v>0.007499557176965373</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00974168648198012</v>
+        <v>0.009741703143452796</v>
       </c>
       <c r="J10" t="n">
-        <v>0.04458887595101676</v>
+        <v>0.04458887592527555</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01190418081690332</v>
+        <v>0.0119041644809008</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.006830362556027613</v>
+        <v>-0.006830359768365832</v>
       </c>
       <c r="M10" t="n">
-        <v>0.0254862592067964</v>
+        <v>0.02548626871709544</v>
       </c>
     </row>
     <row r="11">
@@ -1168,40 +1168,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.03339262578189272</v>
+        <v>0.03339258820560981</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02827015146920691</v>
+        <v>0.02827013491248067</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0298825686015476</v>
+        <v>0.029882581141819</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0004806151576768403</v>
+        <v>0.0004806581162570173</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.001106555693483212</v>
+        <v>-0.001106551972723699</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0002776740321931119</v>
+        <v>-0.0002776720455737413</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001881980711318011</v>
+        <v>0.001881975708770497</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0246329029619418</v>
+        <v>0.02463290276657371</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01190418081690332</v>
+        <v>0.0119041644809008</v>
       </c>
       <c r="K11" t="n">
-        <v>0.04274868897782444</v>
+        <v>0.04274865450024606</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.006333867158072055</v>
+        <v>-0.006333851508033089</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03973017892135465</v>
+        <v>0.03973014884462577</v>
       </c>
     </row>
     <row r="12">
@@ -1211,40 +1211,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.006984632648182314</v>
+        <v>-0.006984614515524904</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.006923672132899366</v>
+        <v>-0.006923664159927042</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.007008072402308412</v>
+        <v>-0.007008057251556645</v>
       </c>
       <c r="E12" t="n">
-        <v>0.00576142691507104</v>
+        <v>0.00576139837511575</v>
       </c>
       <c r="F12" t="n">
-        <v>0.004361811919052664</v>
+        <v>0.004361823878065251</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006216706243753326</v>
+        <v>0.006216703894578712</v>
       </c>
       <c r="H12" t="n">
-        <v>0.005267436496113646</v>
+        <v>0.005267434459916362</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.001700713036666564</v>
+        <v>-0.001700713853494101</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.006830362556027613</v>
+        <v>-0.006830359768365832</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.006333867158072055</v>
+        <v>-0.006333851508033089</v>
       </c>
       <c r="L12" t="n">
-        <v>0.02237618985940767</v>
+        <v>0.02237612888293778</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.01025756880625418</v>
+        <v>-0.01025756571745604</v>
       </c>
     </row>
     <row r="13">
@@ -1254,40 +1254,40 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.03677496618860314</v>
+        <v>0.03677495510865</v>
       </c>
       <c r="C13" t="n">
-        <v>0.04051506590783106</v>
+        <v>0.04051506380915469</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04655603178803784</v>
+        <v>0.04655606142444107</v>
       </c>
       <c r="E13" t="n">
-        <v>4.016612443580877e-05</v>
+        <v>4.019200736346342e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.001505117009196318</v>
+        <v>-0.001505125204721985</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0001213940806772489</v>
+        <v>0.0001214081698984464</v>
       </c>
       <c r="H13" t="n">
-        <v>0.01259465896827418</v>
+        <v>0.0125946562048136</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0310536900294825</v>
+        <v>0.03105372179720148</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0254862592067964</v>
+        <v>0.02548626871709544</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03973017892135465</v>
+        <v>0.03973014884462577</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.01025756880625418</v>
+        <v>-0.01025756571745604</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1179573219649314</v>
+        <v>0.1179573360243339</v>
       </c>
     </row>
   </sheetData>

</xml_diff>